<commit_message>
Update public roster from sign sheet
</commit_message>
<xml_diff>
--- a/app/data/sign.xlsx
+++ b/app/data/sign.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Xindian_Cup\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BADAAFC3-68B0-4468-8620-92D577566514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72511171-C023-4169-B7B1-441585AE8438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="96">
   <si>
     <t>1. 隊名</t>
   </si>
@@ -241,13 +241,86 @@
   </si>
   <si>
     <t>陳詠心</t>
+  </si>
+  <si>
+    <t>新店膨魚晏</t>
+  </si>
+  <si>
+    <t>劉錫安</t>
+  </si>
+  <si>
+    <t>andy99663399</t>
+  </si>
+  <si>
+    <t>andy99663390@gmail.com</t>
+  </si>
+  <si>
+    <t>諸政豪</t>
+  </si>
+  <si>
+    <t>黃建宸</t>
+  </si>
+  <si>
+    <t>吳宜霖</t>
+  </si>
+  <si>
+    <t>林晏如</t>
+  </si>
+  <si>
+    <t>張詩筠</t>
+  </si>
+  <si>
+    <t>還沒確定</t>
+  </si>
+  <si>
+    <t>17+</t>
+  </si>
+  <si>
+    <t>施中堂</t>
+  </si>
+  <si>
+    <t>tommy10815</t>
+  </si>
+  <si>
+    <t>a5305tommy@gmail.com</t>
+  </si>
+  <si>
+    <t>陳沅禾</t>
+  </si>
+  <si>
+    <t>王德翰</t>
+  </si>
+  <si>
+    <t>宋曼寧</t>
+  </si>
+  <si>
+    <t>宋曼甄</t>
+  </si>
+  <si>
+    <t>洪詩婷</t>
+  </si>
+  <si>
+    <t>吳珊菱</t>
+  </si>
+  <si>
+    <t>曾韻如</t>
+  </si>
+  <si>
+    <t>李佳鴻</t>
+  </si>
+  <si>
+    <t>想到再加</t>
+  </si>
+  <si>
+    <t>阿邊</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -278,6 +351,12 @@
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Microsoft JhengHei"/>
+      <charset val="136"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -305,7 +384,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -478,11 +557,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFF8F9FA"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF442F65"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFF8F9FA"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -530,6 +639,24 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -812,10 +939,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AE7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:30" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" ht="27" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -907,7 +1034,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" ht="53.4" thickBot="1">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -999,7 +1126,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:30" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" ht="53.4" thickBot="1">
       <c r="A3" s="9" t="s">
         <v>34</v>
       </c>
@@ -1091,7 +1218,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:30" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" ht="53.4" thickBot="1">
       <c r="A4" s="12" t="s">
         <v>48</v>
       </c>
@@ -1146,8 +1273,8 @@
       <c r="R4" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="S4" s="6" t="s">
-        <v>57</v>
+      <c r="S4" s="22" t="s">
+        <v>95</v>
       </c>
       <c r="T4" s="6" t="s">
         <v>33</v>
@@ -1183,7 +1310,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:30" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" ht="53.4" thickBot="1">
       <c r="A5" s="13" t="s">
         <v>58</v>
       </c>
@@ -1274,6 +1401,192 @@
       <c r="AD5" s="16" t="s">
         <v>33</v>
       </c>
+    </row>
+    <row r="6" spans="1:31" ht="15.6" thickBot="1">
+      <c r="A6" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="L6" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="N6" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="O6" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="P6" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q6" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="R6" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="S6" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="T6" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="U6" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="V6" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="W6" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="X6" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y6" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="Z6" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA6" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="AB6" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC6" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="AD6" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE6" s="18"/>
+    </row>
+    <row r="7" spans="1:31" ht="15.6" thickBot="1">
+      <c r="A7" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="H7" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="J7" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="K7" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="L7" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="M7" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="N7" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="O7" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="P7" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q7" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="R7" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="S7" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="T7" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="U7" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="V7" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="W7" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="X7" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y7" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="Z7" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA7" s="20">
+        <v>17</v>
+      </c>
+      <c r="AB7" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC7" s="20">
+        <v>17</v>
+      </c>
+      <c r="AD7" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE7" s="21"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
Sync public roster from updated sign sheet
</commit_message>
<xml_diff>
--- a/app/data/sign.xlsx
+++ b/app/data/sign.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Xindian_Cup\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72511171-C023-4169-B7B1-441585AE8438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC38551A-F79B-4AC5-9B10-B01500A3347E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="112">
   <si>
     <t>1. 隊名</t>
   </si>
@@ -314,13 +314,61 @@
   <si>
     <t>阿邊</t>
     <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>新店溪畔1.1</t>
+  </si>
+  <si>
+    <t>陳珖萭</t>
+  </si>
+  <si>
+    <t>timmy71630</t>
+  </si>
+  <si>
+    <t>timmy81630@gmail.com</t>
+  </si>
+  <si>
+    <t>單大誠</t>
+  </si>
+  <si>
+    <t>劉采靈</t>
+  </si>
+  <si>
+    <t>胡孝新</t>
+  </si>
+  <si>
+    <t>褚凡瑋</t>
+  </si>
+  <si>
+    <t>沈容軒</t>
+  </si>
+  <si>
+    <t>王又禾</t>
+  </si>
+  <si>
+    <t>黃紹傑</t>
+  </si>
+  <si>
+    <t>李思諭</t>
+  </si>
+  <si>
+    <t>欣妤</t>
+  </si>
+  <si>
+    <t>劉錫忠</t>
+  </si>
+  <si>
+    <t>周莉雯</t>
+  </si>
+  <si>
+    <t>後補</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -357,6 +405,12 @@
       <name val="Microsoft JhengHei"/>
       <charset val="136"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -384,7 +438,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -439,21 +493,6 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="FFFFFFFF"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFFFFFFF"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFF8F9FA"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
         <color rgb="FFCCCCCC"/>
       </left>
       <right style="medium">
@@ -484,21 +523,6 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="FFF8F9FA"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFF8F9FA"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFF8F9FA"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
         <color rgb="FFCCCCCC"/>
       </left>
       <right style="medium">
@@ -509,51 +533,6 @@
       </top>
       <bottom style="medium">
         <color rgb="FFF8F9FA"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFF8F9FA"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFF8F9FA"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF442F65"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFF8F9FA"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF442F65"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF442F65"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF442F65"/>
       </bottom>
       <diagonal/>
     </border>
@@ -587,11 +566,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF8F9FA"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFF8F9FA"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -605,59 +599,33 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -939,7 +907,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:31" ht="27" thickBot="1">
@@ -1034,559 +1002,652 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="53.4" thickBot="1">
-      <c r="A2" s="5">
+    <row r="2" spans="1:31" ht="15.6" thickBot="1">
+      <c r="A2" s="14">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" s="7">
+      <c r="F2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" s="14">
         <v>1</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" s="7">
+      <c r="H2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="14">
         <v>1</v>
       </c>
-      <c r="J2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="K2" s="7">
+      <c r="J2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="14">
         <v>1</v>
       </c>
-      <c r="L2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="M2" s="7">
+      <c r="L2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" s="14">
         <v>1</v>
       </c>
-      <c r="N2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" s="7">
+      <c r="N2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="O2" s="14">
         <v>1</v>
       </c>
-      <c r="P2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q2" s="7">
+      <c r="P2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q2" s="14">
         <v>1</v>
       </c>
-      <c r="R2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="S2" s="7">
+      <c r="R2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="S2" s="14">
         <v>1</v>
       </c>
-      <c r="T2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="U2" s="7">
+      <c r="T2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="U2" s="14">
         <v>1</v>
       </c>
-      <c r="V2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="W2" s="7">
+      <c r="V2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="W2" s="14">
         <v>1</v>
       </c>
-      <c r="X2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y2" s="7">
+      <c r="X2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y2" s="14">
         <v>1</v>
       </c>
-      <c r="Z2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA2" s="7">
+      <c r="Z2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA2" s="14">
         <v>1</v>
       </c>
-      <c r="AB2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC2" s="7">
+      <c r="AB2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC2" s="14">
         <v>1</v>
       </c>
-      <c r="AD2" s="8" t="s">
+      <c r="AD2" s="14" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="53.4" thickBot="1">
-      <c r="A3" s="9" t="s">
+    <row r="3" spans="1:31" ht="15.6" thickBot="1">
+      <c r="A3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="5">
         <v>919566724</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" s="10" t="s">
+      <c r="F3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" s="10" t="s">
+      <c r="H3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="K3" s="10" t="s">
+      <c r="J3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K3" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="L3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="M3" s="10" t="s">
+      <c r="L3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M3" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="N3" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="O3" s="10" t="s">
+      <c r="N3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="O3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="P3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q3" s="10" t="s">
+      <c r="P3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q3" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="R3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="S3" s="10" t="s">
+      <c r="R3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="S3" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="T3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="U3" s="10" t="s">
+      <c r="T3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="V3" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="W3" s="10" t="s">
+      <c r="V3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="W3" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="X3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y3" s="10" t="s">
+      <c r="X3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y3" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="Z3" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA3" s="10" t="s">
+      <c r="Z3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA3" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="AB3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC3" s="10" t="s">
+      <c r="AB3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC3" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="AD3" s="11" t="s">
+      <c r="AD3" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="53.4" thickBot="1">
-      <c r="A4" s="12" t="s">
+    <row r="4" spans="1:31" ht="15.6" thickBot="1">
+      <c r="A4" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" s="6" t="s">
+      <c r="F4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="I4" s="6" t="s">
+      <c r="H4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="K4" s="6" t="s">
+      <c r="J4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="L4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="6" t="s">
+      <c r="L4" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="M4" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="N4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O4" s="6" t="s">
+      <c r="N4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="O4" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="P4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q4" s="6" t="s">
+      <c r="P4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q4" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="R4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="S4" s="22" t="s">
+      <c r="R4" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="S4" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="T4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="U4" s="6" t="s">
+      <c r="T4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="U4" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="V4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="W4" s="6" t="s">
+      <c r="V4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="W4" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="X4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y4" s="6" t="s">
+      <c r="X4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y4" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="Z4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA4" s="6" t="s">
+      <c r="Z4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA4" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="AB4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC4" s="6" t="s">
+      <c r="AB4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC4" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="AD4" s="8" t="s">
+      <c r="AD4" s="14" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:31" ht="53.4" thickBot="1">
-      <c r="A5" s="13" t="s">
+    <row r="5" spans="1:31" ht="15.6" thickBot="1">
+      <c r="A5" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="F5" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="14" t="s">
+      <c r="F5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" s="14" t="s">
+      <c r="H5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="J5" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="K5" s="14" t="s">
+      <c r="J5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K5" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="L5" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="M5" s="14" t="s">
+      <c r="L5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M5" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="N5" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="O5" s="14" t="s">
+      <c r="N5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O5" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="P5" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q5" s="14" t="s">
+      <c r="P5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q5" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="R5" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="S5" s="14" t="s">
+      <c r="R5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="S5" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="T5" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="U5" s="14" t="s">
+      <c r="T5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="U5" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="V5" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="W5" s="14" t="s">
+      <c r="V5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="W5" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="X5" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y5" s="14" t="s">
+      <c r="X5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y5" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="Z5" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA5" s="15">
+      <c r="Z5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA5" s="5">
         <v>123</v>
       </c>
-      <c r="AB5" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC5" s="15">
+      <c r="AB5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC5" s="5">
         <v>123</v>
       </c>
-      <c r="AD5" s="16" t="s">
+      <c r="AD5" s="5" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="F6" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" s="17" t="s">
+      <c r="F6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="17" t="s">
+      <c r="H6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="J6" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="K6" s="17" t="s">
+      <c r="J6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L6" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="M6" s="17" t="s">
+      <c r="L6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="O6" s="17" t="s">
+      <c r="N6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="O6" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="P6" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q6" s="17" t="s">
+      <c r="P6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q6" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="R6" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="S6" s="17" t="s">
+      <c r="R6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="S6" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="T6" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="U6" s="17" t="s">
+      <c r="T6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="U6" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="V6" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="W6" s="17" t="s">
+      <c r="V6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="W6" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="X6" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y6" s="17" t="s">
+      <c r="X6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y6" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="Z6" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA6" s="17" t="s">
+      <c r="Z6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA6" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="AB6" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC6" s="17" t="s">
+      <c r="AB6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC6" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="AD6" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="AE6" s="18"/>
+      <c r="AD6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE6" s="6"/>
     </row>
     <row r="7" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F7" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="19" t="s">
+      <c r="F7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="H7" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="I7" s="19" t="s">
+      <c r="H7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="J7" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="K7" s="19" t="s">
+      <c r="J7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="K7" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="L7" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="M7" s="19" t="s">
+      <c r="L7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M7" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="N7" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="O7" s="19" t="s">
+      <c r="N7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="O7" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="P7" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q7" s="19" t="s">
+      <c r="P7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q7" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="R7" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="S7" s="19" t="s">
+      <c r="R7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="S7" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="T7" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="U7" s="19" t="s">
+      <c r="T7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="U7" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="V7" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="W7" s="19" t="s">
+      <c r="V7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="W7" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="X7" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y7" s="19" t="s">
+      <c r="X7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y7" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="Z7" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA7" s="20">
+      <c r="Z7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA7" s="8">
         <v>17</v>
       </c>
-      <c r="AB7" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="AC7" s="20">
+      <c r="AB7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC7" s="8">
         <v>17</v>
       </c>
-      <c r="AD7" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="AE7" s="21"/>
+      <c r="AD7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE7" s="9"/>
+    </row>
+    <row r="8" spans="1:31" ht="16.2" thickBot="1">
+      <c r="A8" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="N8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="O8" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="P8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q8" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="R8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="S8" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="T8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="U8" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="V8" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="W8" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="X8" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y8" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="Z8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA8" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="AB8" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC8" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD8" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE8" s="13"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
Update roster and remove test suite
</commit_message>
<xml_diff>
--- a/app/data/sign.xlsx
+++ b/app/data/sign.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Xindian_Cup\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC38551A-F79B-4AC5-9B10-B01500A3347E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A158C4CC-7CC3-4C53-9D67-507825AAA762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28800" yWindow="1440" windowWidth="27000" windowHeight="14040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="126">
   <si>
     <t>1. 隊名</t>
   </si>
@@ -362,13 +362,58 @@
   </si>
   <si>
     <t>後補</t>
+  </si>
+  <si>
+    <t>蘇宣豪</t>
+  </si>
+  <si>
+    <t>pk2914su</t>
+  </si>
+  <si>
+    <t>pk2914su@gmail.com</t>
+  </si>
+  <si>
+    <t>徐達希</t>
+  </si>
+  <si>
+    <t>徐培勳</t>
+  </si>
+  <si>
+    <t>徐羽彤</t>
+  </si>
+  <si>
+    <t>萬礎榮</t>
+  </si>
+  <si>
+    <t>陳昭榮</t>
+  </si>
+  <si>
+    <t>李雅婷</t>
+  </si>
+  <si>
+    <t>梁孝傑</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>補</t>
+  </si>
+  <si>
+    <t>老馬一中</t>
+  </si>
+  <si>
+    <t>徐魁谷</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>梁智華</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -410,6 +455,19 @@
       <color rgb="FF222222"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Microsoft JhengHei"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Microsoft JhengHei"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -585,7 +643,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -626,6 +684,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -907,8 +977,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="28.875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="27" thickBot="1">
       <c r="A1" s="1" t="s">
@@ -1648,6 +1721,99 @@
         <v>41</v>
       </c>
       <c r="AE8" s="13"/>
+    </row>
+    <row r="9" spans="1:31" ht="40.200000000000003" thickBot="1">
+      <c r="A9" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="J9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K9" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="M9" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="N9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="O9" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="P9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q9" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="R9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="S9" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="T9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="U9" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="V9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="W9" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="X9" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y9" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="Z9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA9" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="AB9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC9" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="AD9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE9" s="17"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
Update roster from latest signup sheet
</commit_message>
<xml_diff>
--- a/app/data/sign.xlsx
+++ b/app/data/sign.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Xindian_Cup\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A158C4CC-7CC3-4C53-9D67-507825AAA762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EC0E03-CC99-4E55-96E0-47296EE4210D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="1440" windowWidth="27000" windowHeight="14040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="130">
   <si>
     <t>1. 隊名</t>
   </si>
@@ -407,13 +407,25 @@
   <si>
     <t>梁智華</t>
     <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>寄送狀態</t>
+  </si>
+  <si>
+    <t>已寄送</t>
+  </si>
+  <si>
+    <t>曾能祐</t>
+  </si>
+  <si>
+    <t>鍾宜庭</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -469,6 +481,13 @@
       <name val="Microsoft JhengHei"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -496,27 +515,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF5B3F86"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF5B3F86"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF442F65"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF442F65"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -643,58 +647,61 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -983,837 +990,860 @@
     <col min="1" max="1" width="28.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="27" thickBot="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:31" ht="15.6" thickBot="1">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="V1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="X1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Y1" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AA1" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AB1" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AC1" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="4" t="s">
+      <c r="AD1" s="16" t="s">
         <v>29</v>
+      </c>
+      <c r="AE1" s="17" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A2" s="14">
+      <c r="A2" s="10">
         <v>1</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" s="14">
+      <c r="F2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" s="10">
         <v>1</v>
       </c>
-      <c r="H2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" s="14">
+      <c r="H2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="10">
         <v>1</v>
       </c>
-      <c r="J2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="K2" s="14">
+      <c r="J2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="10">
         <v>1</v>
       </c>
-      <c r="L2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="M2" s="14">
+      <c r="L2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" s="10">
         <v>1</v>
       </c>
-      <c r="N2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" s="14">
+      <c r="N2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="O2" s="10">
         <v>1</v>
       </c>
-      <c r="P2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q2" s="14">
+      <c r="P2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q2" s="10">
         <v>1</v>
       </c>
-      <c r="R2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="S2" s="14">
+      <c r="R2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="S2" s="10">
         <v>1</v>
       </c>
-      <c r="T2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="U2" s="14">
+      <c r="T2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="U2" s="10">
         <v>1</v>
       </c>
-      <c r="V2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="W2" s="14">
+      <c r="V2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="W2" s="10">
         <v>1</v>
       </c>
-      <c r="X2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y2" s="14">
+      <c r="X2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y2" s="10">
         <v>1</v>
       </c>
-      <c r="Z2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA2" s="14">
+      <c r="Z2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA2" s="10">
         <v>1</v>
       </c>
-      <c r="AB2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC2" s="14">
+      <c r="AB2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC2" s="10">
         <v>1</v>
       </c>
-      <c r="AD2" s="14" t="s">
-        <v>33</v>
+      <c r="AD2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE2" s="18" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="1">
         <v>919566724</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" s="5" t="s">
+      <c r="H3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K3" s="5" t="s">
+      <c r="J3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M3" s="5" t="s">
+      <c r="L3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="M3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="N3" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="O3" s="5" t="s">
+      <c r="N3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="P3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q3" s="5" t="s">
+      <c r="P3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q3" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="R3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="S3" s="5" t="s">
+      <c r="R3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="T3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="U3" s="5" t="s">
+      <c r="T3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="V3" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="W3" s="5" t="s">
+      <c r="V3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="W3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="X3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y3" s="5" t="s">
+      <c r="X3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="Z3" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA3" s="5" t="s">
+      <c r="Z3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AB3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC3" s="5" t="s">
+      <c r="AB3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AD3" s="5" t="s">
-        <v>33</v>
+      <c r="AD3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE3" s="2" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" s="14" t="s">
+      <c r="F4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="I4" s="14" t="s">
+      <c r="H4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="K4" s="14" t="s">
+      <c r="J4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="L4" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="14" t="s">
+      <c r="L4" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="M4" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="N4" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="O4" s="14" t="s">
+      <c r="N4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="O4" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="P4" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q4" s="14" t="s">
+      <c r="P4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="R4" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="S4" s="10" t="s">
+      <c r="R4" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="S4" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="T4" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="U4" s="14" t="s">
+      <c r="T4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U4" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="V4" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="W4" s="14" t="s">
+      <c r="V4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="W4" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="X4" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y4" s="14" t="s">
+      <c r="X4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y4" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="Z4" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA4" s="14" t="s">
+      <c r="Z4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA4" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="AB4" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC4" s="14" t="s">
+      <c r="AB4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC4" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="AD4" s="14" t="s">
-        <v>33</v>
+      <c r="AD4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE4" s="18" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" s="5" t="s">
+      <c r="H5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="J5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K5" s="5" t="s">
+      <c r="J5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="L5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M5" s="5" t="s">
+      <c r="L5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="M5" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="N5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O5" s="5" t="s">
+      <c r="N5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="P5" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q5" s="5" t="s">
+      <c r="P5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="R5" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="S5" s="5" t="s">
+      <c r="R5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="S5" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="T5" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="U5" s="5" t="s">
+      <c r="T5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U5" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="V5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="W5" s="5" t="s">
+      <c r="V5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="W5" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="X5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y5" s="5" t="s">
+      <c r="X5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y5" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="Z5" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA5" s="5">
+      <c r="Z5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA5" s="1">
         <v>123</v>
       </c>
-      <c r="AB5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC5" s="5">
+      <c r="AB5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC5" s="1">
         <v>123</v>
       </c>
-      <c r="AD5" s="5" t="s">
-        <v>33</v>
+      <c r="AD5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE5" s="2" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="5" t="s">
+      <c r="H6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="J6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K6" s="5" t="s">
+      <c r="J6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="L6" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="M6" s="5" t="s">
+      <c r="L6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="O6" s="5" t="s">
+      <c r="N6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O6" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="P6" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q6" s="5" t="s">
+      <c r="P6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="R6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="S6" s="5" t="s">
+      <c r="R6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="T6" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="U6" s="5" t="s">
+      <c r="T6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="V6" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="W6" s="5" t="s">
+      <c r="V6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="W6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="X6" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y6" s="5" t="s">
+      <c r="X6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="Z6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA6" s="5" t="s">
+      <c r="Z6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="AB6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC6" s="5" t="s">
+      <c r="AB6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="AD6" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="AE6" s="6"/>
+      <c r="AD6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE6" s="2" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="7" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="7" t="s">
+      <c r="F7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="I7" s="7" t="s">
+      <c r="H7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="J7" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K7" s="7" t="s">
+      <c r="J7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="L7" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="M7" s="7" t="s">
+      <c r="L7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M7" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="N7" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="O7" s="7" t="s">
+      <c r="N7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="O7" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="P7" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q7" s="7" t="s">
+      <c r="P7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q7" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="R7" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="S7" s="7" t="s">
+      <c r="R7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="S7" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="T7" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="U7" s="7" t="s">
+      <c r="T7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="U7" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="V7" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="W7" s="7" t="s">
+      <c r="V7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="W7" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="X7" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y7" s="7" t="s">
+      <c r="X7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y7" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="Z7" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA7" s="8">
+      <c r="Z7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA7" s="4">
         <v>17</v>
       </c>
-      <c r="AB7" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AC7" s="8">
+      <c r="AB7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC7" s="4">
         <v>17</v>
       </c>
-      <c r="AD7" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AE7" s="9"/>
+      <c r="AD7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE7" s="5" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="8" spans="1:31" ht="16.2" thickBot="1">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="F8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8" s="11" t="s">
+      <c r="F8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="H8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="I8" s="11" t="s">
+      <c r="H8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="J8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="K8" s="11" t="s">
+      <c r="J8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="K8" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="L8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="M8" s="11" t="s">
+      <c r="L8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M8" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="N8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="O8" s="11" t="s">
+      <c r="N8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="O8" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="P8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q8" s="11" t="s">
+      <c r="P8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q8" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="R8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="S8" s="11" t="s">
+      <c r="R8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S8" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="T8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="U8" s="11" t="s">
+      <c r="T8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="U8" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="V8" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="W8" s="11" t="s">
+      <c r="V8" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="W8" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="X8" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y8" s="11" t="s">
+      <c r="X8" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y8" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="Z8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA8" s="12" t="s">
+      <c r="Z8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA8" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="AB8" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="AC8" s="11" t="s">
+      <c r="AB8" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC8" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="AD8" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="AE8" s="13"/>
+      <c r="AD8" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE8" s="9" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="9" spans="1:31" ht="40.200000000000003" thickBot="1">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="F9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="G9" s="15" t="s">
+      <c r="F9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="H9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" s="15" t="s">
+      <c r="H9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="J9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="K9" s="15" t="s">
+      <c r="J9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="K9" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="L9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="M9" s="15" t="s">
+      <c r="L9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="M9" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="N9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="O9" s="15" t="s">
+      <c r="N9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="O9" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="P9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q9" s="15" t="s">
+      <c r="P9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q9" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="R9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="S9" s="16" t="s">
+      <c r="R9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="S9" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="T9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="U9" s="18" t="s">
+      <c r="T9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="U9" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="V9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="W9" s="18" t="s">
+      <c r="V9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="W9" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="X9" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y9" s="15" t="s">
+      <c r="X9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y9" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="Z9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA9" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="AB9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC9" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="Z9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA9" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="AB9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC9" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="AD9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="AE9" s="17"/>
+      <c r="AD9" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE9" s="13" t="s">
+        <v>127</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
Update first team roster
</commit_message>
<xml_diff>
--- a/app/data/sign.xlsx
+++ b/app/data/sign.xlsx
@@ -1,31 +1,43 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Xindian_Cup\app\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EC0E03-CC99-4E55-96E0-47296EE4210D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="工作表1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>工作表</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>工作表1</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="130">
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>user</dc:creator>
+  <cp:lastModifiedBy>user</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2015-06-05T18:19:34Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-04-28T06:32:01Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="142">
   <si>
     <t>1. 隊名</t>
   </si>
@@ -419,11 +431,47 @@
   </si>
   <si>
     <t>鍾宜庭</t>
+  </si>
+  <si>
+    <t>玻璃心又玻璃膝</t>
+  </si>
+  <si>
+    <t>陳柏諺</t>
+  </si>
+  <si>
+    <t>唐翰霖</t>
+  </si>
+  <si>
+    <t>張尚橙</t>
+  </si>
+  <si>
+    <t>陳可軒</t>
+  </si>
+  <si>
+    <t>吳玟靜</t>
+  </si>
+  <si>
+    <t>蕭志晴</t>
+  </si>
+  <si>
+    <t>林秀俐</t>
+  </si>
+  <si>
+    <t>鄭宇恩</t>
+  </si>
+  <si>
+    <t>李孟芸</t>
+  </si>
+  <si>
+    <t>葉芷妤</t>
+  </si>
+  <si>
+    <t>後續有補跟你說</t>
   </si>
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="10">
     <font>
@@ -721,7 +769,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -982,7 +1030,32 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Xindian_Cup\app\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EC0E03-CC99-4E55-96E0-47296EE4210D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="工作表1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="162913"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AE9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1086,8 +1159,8 @@
       </c>
     </row>
     <row r="2" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A2" s="10">
-        <v>1</v>
+      <c r="A2" s="10" t="s">
+        <v>130</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>30</v>
@@ -1104,78 +1177,72 @@
       <c r="F2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="G2" s="10">
-        <v>1</v>
+      <c r="G2" s="10" t="s">
+        <v>131</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I2" s="10">
-        <v>1</v>
+      <c r="I2" s="10" t="s">
+        <v>132</v>
       </c>
       <c r="J2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="10">
-        <v>1</v>
+      <c r="K2" s="10" t="s">
+        <v>133</v>
       </c>
       <c r="L2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="M2" s="10">
-        <v>1</v>
+      <c r="M2" s="10" t="s">
+        <v>134</v>
       </c>
       <c r="N2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="O2" s="10">
-        <v>1</v>
+      <c r="O2" s="10" t="s">
+        <v>135</v>
       </c>
       <c r="P2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="Q2" s="10">
-        <v>1</v>
+      <c r="Q2" s="10" t="s">
+        <v>136</v>
       </c>
       <c r="R2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="S2" s="10">
-        <v>1</v>
+      <c r="S2" s="10" t="s">
+        <v>137</v>
       </c>
       <c r="T2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="U2" s="10">
-        <v>1</v>
+      <c r="U2" s="10" t="s">
+        <v>138</v>
       </c>
       <c r="V2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="W2" s="10">
-        <v>1</v>
+        <v>41</v>
+      </c>
+      <c r="W2" s="10" t="s">
+        <v>139</v>
       </c>
       <c r="X2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y2" s="10">
-        <v>1</v>
+        <v>41</v>
+      </c>
+      <c r="Y2" s="10" t="s">
+        <v>140</v>
       </c>
       <c r="Z2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA2" s="10">
-        <v>1</v>
-      </c>
-      <c r="AB2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC2" s="10">
-        <v>1</v>
-      </c>
-      <c r="AD2" s="10" t="s">
-        <v>33</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="AA2" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="AB2" s="10"/>
+      <c r="AC2" s="10"/>
+      <c r="AD2" s="10"/>
       <c r="AE2" s="18" t="s">
         <v>127</v>
       </c>

</xml_diff>

<commit_message>
Sync team roster updates
</commit_message>
<xml_diff>
--- a/app/data/sign.xlsx
+++ b/app/data/sign.xlsx
@@ -1,43 +1,31 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>Microsoft Excel</Application>
-  <DocSecurity>0</DocSecurity>
-  <ScaleCrop>false</ScaleCrop>
-  <HeadingPairs>
-    <vt:vector size="2" baseType="variant">
-      <vt:variant>
-        <vt:lpstr>工作表</vt:lpstr>
-      </vt:variant>
-      <vt:variant>
-        <vt:i4>1</vt:i4>
-      </vt:variant>
-    </vt:vector>
-  </HeadingPairs>
-  <TitlesOfParts>
-    <vt:vector size="1" baseType="lpstr">
-      <vt:lpstr>工作表1</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-  <Company/>
-  <LinksUpToDate>false</LinksUpToDate>
-  <SharedDoc>false</SharedDoc>
-  <HyperlinksChanged>false</HyperlinksChanged>
-  <AppVersion>16.0300</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kenny\Desktop\Xindian_Cup\app\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A8065D9-76F4-4FE6-BDB8-9195CB92B02A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="工作表1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="162913"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <dc:creator>user</dc:creator>
-  <cp:lastModifiedBy>user</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2015-06-05T18:19:34Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-04-28T06:32:01Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="142">
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="145">
   <si>
     <t>1. 隊名</t>
   </si>
@@ -467,11 +455,23 @@
   </si>
   <si>
     <t>後續有補跟你說</t>
+  </si>
+  <si>
+    <t>胡采妮</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>褚婕</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>王善豪</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="10">
     <font>
@@ -563,7 +563,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -691,11 +691,78 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF8F9FA"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF442F65"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF8F9FA"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF442F65"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -703,15 +770,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -719,9 +777,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -751,6 +806,31 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -769,7 +849,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1030,224 +1110,199 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Xindian_Cup\app\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EC0E03-CC99-4E55-96E0-47296EE4210D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="工作表1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AE9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="28.875" customWidth="1"/>
+    <col min="1" max="1" width="28.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:31" ht="16.5" thickBot="1">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="K1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="L1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="N1" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="O1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="P1" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="Q1" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="16" t="s">
+      <c r="R1" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="16" t="s">
+      <c r="S1" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="16" t="s">
+      <c r="T1" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="16" t="s">
+      <c r="U1" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="16" t="s">
+      <c r="V1" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="16" t="s">
+      <c r="W1" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="16" t="s">
+      <c r="X1" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="16" t="s">
+      <c r="Y1" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="16" t="s">
+      <c r="Z1" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="16" t="s">
+      <c r="AA1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="16" t="s">
+      <c r="AB1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="16" t="s">
+      <c r="AC1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="16" t="s">
+      <c r="AD1" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="17" t="s">
+      <c r="AE1" s="13" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:31" ht="16.5" thickBot="1">
+      <c r="A2" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" s="10" t="s">
+      <c r="F2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="H2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" s="10" t="s">
+      <c r="H2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="J2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="K2" s="10" t="s">
+      <c r="J2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="L2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="M2" s="10" t="s">
+      <c r="L2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="N2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" s="10" t="s">
+      <c r="N2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="O2" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="P2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q2" s="10" t="s">
+      <c r="P2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q2" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="R2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="S2" s="10" t="s">
+      <c r="R2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="S2" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="T2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="U2" s="10" t="s">
+      <c r="T2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="U2" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="V2" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="W2" s="10" t="s">
+      <c r="V2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="W2" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="X2" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y2" s="10" t="s">
+      <c r="X2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y2" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="Z2" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA2" s="10" t="s">
+      <c r="Z2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA2" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="AB2" s="10"/>
-      <c r="AC2" s="10"/>
-      <c r="AD2" s="10"/>
-      <c r="AE2" s="18" t="s">
+      <c r="AB2" s="6"/>
+      <c r="AC2" s="6"/>
+      <c r="AD2" s="6"/>
+      <c r="AE2" s="14" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="15.6" thickBot="1">
+    <row r="3" spans="1:31" ht="16.5" thickBot="1">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
@@ -1342,573 +1397,573 @@
         <v>127</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:31" ht="16.5" thickBot="1">
+      <c r="A4" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" s="10" t="s">
+      <c r="F4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I4" s="10" t="s">
+      <c r="H4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="K4" s="10" t="s">
+      <c r="J4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="L4" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="10" t="s">
+      <c r="L4" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M4" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="N4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="O4" s="10" t="s">
+      <c r="N4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="O4" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="P4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q4" s="10" t="s">
+      <c r="P4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q4" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="R4" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="S4" s="6" t="s">
+      <c r="R4" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="S4" s="3" t="s">
         <v>95</v>
       </c>
       <c r="T4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="U4" s="10" t="s">
+      <c r="U4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="V4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="W4" s="10" t="s">
+      <c r="V4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="W4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="X4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y4" s="10" t="s">
+      <c r="X4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="Z4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA4" s="10" t="s">
+      <c r="Z4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="AB4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC4" s="10" t="s">
+      <c r="AB4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="AD4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="AE4" s="18" t="s">
+      <c r="AD4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE4" s="14" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:31" ht="16.5" thickBot="1">
+      <c r="A5" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="1" t="s">
+      <c r="F5" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" s="1" t="s">
+      <c r="H5" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="K5" s="1" t="s">
+      <c r="J5" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="K5" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="L5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="M5" s="1" t="s">
+      <c r="L5" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="M5" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="N5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O5" s="1" t="s">
+      <c r="N5" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="O5" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="P5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q5" s="1" t="s">
+      <c r="P5" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q5" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="R5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S5" s="1" t="s">
+      <c r="R5" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="S5" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="T5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="U5" s="1" t="s">
+      <c r="T5" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="U5" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="V5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="W5" s="1" t="s">
+      <c r="V5" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="W5" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="X5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y5" s="1" t="s">
+      <c r="X5" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y5" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="Z5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA5" s="1">
+      <c r="Z5" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA5" s="16">
         <v>123</v>
       </c>
-      <c r="AB5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC5" s="1">
+      <c r="AB5" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC5" s="16">
         <v>123</v>
       </c>
-      <c r="AD5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AE5" s="2" t="s">
+      <c r="AD5" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE5" s="17" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="6" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:31" s="21" customFormat="1" ht="16.5" thickBot="1">
+      <c r="A6" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" s="1" t="s">
+      <c r="F6" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="1" t="s">
+      <c r="H6" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="K6" s="1" t="s">
+      <c r="J6" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="K6" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="L6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M6" s="1" t="s">
+      <c r="L6" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O6" s="1" t="s">
+      <c r="N6" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="O6" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="P6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q6" s="1" t="s">
+      <c r="P6" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q6" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="R6" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="S6" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="T6" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="U6" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="V6" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="W6" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="X6" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y6" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="R6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="S6" s="1" t="s">
+      <c r="Z6" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA6" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="T6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="U6" s="1" t="s">
+      <c r="AB6" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC6" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="V6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="W6" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="X6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y6" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="Z6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA6" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="AB6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC6" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="AD6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AE6" s="2" t="s">
+      <c r="AD6" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE6" s="20" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="7" spans="1:31" ht="15.6" thickBot="1">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:31" s="21" customFormat="1" ht="16.5" thickBot="1">
+      <c r="A7" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="3" t="s">
+      <c r="F7" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="H7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="I7" s="3" t="s">
+      <c r="H7" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="J7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="K7" s="3" t="s">
+      <c r="J7" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="K7" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="L7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M7" s="3" t="s">
+      <c r="L7" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="M7" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="N7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="O7" s="3" t="s">
+      <c r="N7" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="O7" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="P7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q7" s="3" t="s">
+      <c r="P7" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q7" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="R7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="S7" s="3" t="s">
+      <c r="R7" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="S7" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="T7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="U7" s="3" t="s">
+      <c r="T7" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="U7" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="V7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="W7" s="3" t="s">
+      <c r="V7" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="W7" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="X7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y7" s="3" t="s">
+      <c r="X7" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y7" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="Z7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="AA7" s="4">
+      <c r="Z7" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA7" s="23">
         <v>17</v>
       </c>
-      <c r="AB7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="AC7" s="4">
+      <c r="AB7" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC7" s="23">
         <v>17</v>
       </c>
-      <c r="AD7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="AE7" s="5" t="s">
+      <c r="AD7" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE7" s="22" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="16.2" thickBot="1">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:31" ht="16.5" thickBot="1">
+      <c r="A8" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8" s="7" t="s">
+      <c r="F8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="I8" s="7" t="s">
+      <c r="H8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="J8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K8" s="7" t="s">
+      <c r="J8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="K8" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="L8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="M8" s="7" t="s">
+      <c r="L8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M8" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="N8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="O8" s="7" t="s">
+      <c r="N8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="O8" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="P8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q8" s="7" t="s">
+      <c r="P8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q8" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="R8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="S8" s="7" t="s">
+      <c r="R8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="S8" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="T8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="U8" s="7" t="s">
+      <c r="T8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="U8" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="V8" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="W8" s="7" t="s">
+      <c r="V8" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="W8" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="X8" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y8" s="7" t="s">
+      <c r="X8" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y8" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="Z8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA8" s="8" t="s">
+      <c r="Z8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA8" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="AB8" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AC8" s="7" t="s">
+      <c r="AB8" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC8" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="AD8" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AE8" s="9" t="s">
+      <c r="AD8" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE8" s="19" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="9" spans="1:31" ht="40.200000000000003" thickBot="1">
-      <c r="A9" s="11" t="s">
+    <row r="9" spans="1:31" ht="39" thickBot="1">
+      <c r="A9" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="F9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="G9" s="11" t="s">
+      <c r="F9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="H9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" s="11" t="s">
+      <c r="H9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="J9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="K9" s="11" t="s">
+      <c r="J9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="K9" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="L9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="M9" s="11" t="s">
+      <c r="L9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M9" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="N9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="O9" s="11" t="s">
+      <c r="N9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="O9" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="P9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q9" s="11" t="s">
+      <c r="P9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q9" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="R9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="S9" s="12" t="s">
+      <c r="R9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S9" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="T9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="U9" s="14" t="s">
+      <c r="T9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="U9" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="V9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="W9" s="14" t="s">
+      <c r="V9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="W9" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="X9" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y9" s="19" t="s">
+      <c r="X9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y9" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="Z9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA9" s="19" t="s">
+      <c r="Z9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA9" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="AB9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC9" s="11" t="s">
+      <c r="AB9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC9" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="AD9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="AE9" s="13" t="s">
+      <c r="AD9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE9" s="9" t="s">
         <v>127</v>
       </c>
     </row>

</xml_diff>